<commit_message>
feat: restructuring the sections
</commit_message>
<xml_diff>
--- a/01-equities-performance-analysis/outputs/similarity_measures.xlsx
+++ b/01-equities-performance-analysis/outputs/similarity_measures.xlsx
@@ -429,6 +429,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pair</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Euclidean Distance</t>
@@ -448,17 +453,17 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>DANGCEM - ZENITHBANK</t>
+          <t>DANGCEM - ZENITHB</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.053214160351119</v>
+        <v>1.053214</v>
       </c>
       <c r="C2" t="n">
-        <v>22.21552148733866</v>
+        <v>22.215521</v>
       </c>
       <c r="D2" t="n">
-        <v>0.06640292914819253</v>
+        <v>0.066403</v>
       </c>
     </row>
     <row r="3">
@@ -468,29 +473,29 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.052723383175602</v>
+        <v>1.052723</v>
       </c>
       <c r="C3" t="n">
-        <v>21.7882542948399</v>
+        <v>21.788254</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03361049338537362</v>
+        <v>0.03361</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>ZENITHBANK - GTCO</t>
+          <t>ZENITHB - GTCO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7361799729980283</v>
+        <v>0.7361799999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>17.3104828616912</v>
+        <v>17.310483</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5630252314390379</v>
+        <v>0.563025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>